<commit_message>
Rewrite the run rate note in plain English
The note explained the annualised run rate in the register of an accounting
standard - extrapolates, arithmetic extrapolation, seasonality, known future
commitments - when the point is simple: it doubles two months into twelve and
assumes the rest of the year looks the same.

It now says what the calculation does, what it ignores in words anyone
reading the report will recognise, and ends by telling the reader how much
weight to put on it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CVBAFohBCYXt1ufjTVDiZj
</commit_message>
<xml_diff>
--- a/reporting/audit/CTS - Discretionary Technology Spend - FY2027 YTD.xlsx
+++ b/reporting/audit/CTS - Discretionary Technology Spend - FY2027 YTD.xlsx
@@ -192,7 +192,7 @@
     <t xml:space="preserve">Note 4 - period covered</t>
   </si>
   <si>
-    <t xml:space="preserve">Actual amounts cover 2 months of a twelve month financial year. The annualised run rate column extrapolates the year-to-date actual evenly across twelve months. It is an arithmetic extrapolation only and makes no allowance for seasonality, timing of renewals or known future commitments.</t>
+    <t xml:space="preserve">These figures cover July and August only, which is 2 months of a twelve month year. The annualised run rate column takes what has been spent so far, divides it by 2 and multiplies by twelve, so it assumes the rest of the year looks like the first 2 months. It makes no allowance for quieter or busier periods, for annual renewals that fall due later in the year, or for spending already committed but not yet incurred. Treat it as a rough indicator, not a forecast.</t>
   </si>
   <si>
     <t xml:space="preserve">Supplier analysis</t>
@@ -2652,7 +2652,7 @@
       <c r="H19" s="21"/>
       <c r="I19" s="21"/>
     </row>
-    <row r="20" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>51</v>
       </c>

</xml_diff>